<commit_message>
style: align sms error workbook with import result
</commit_message>
<xml_diff>
--- a/debt-transfer-sms-notification/assets/短信通知_导入错误明细.xlsx
+++ b/debt-transfer-sms-notification/assets/短信通知_导入错误明细.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="错误数据明细" sheetId="1" r:id="R45829305afc44e1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="错误类型说明" sheetId="2" r:id="R15aa8aff5eb94ff5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="错误数据明细" sheetId="1" r:id="R4e0d7ae102d04a58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="错误类型说明" sheetId="2" r:id="Rcb256ac651d44035"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,15 +14,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="2">
+  <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
-      <x:sz val="11"/>
-      <x:color rgb="FFFFFFFF"/>
+      <x:sz val="10"/>
+      <x:color rgb="FF3F3F3F"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF202B38"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
@@ -35,17 +40,45 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF1677FF"/>
+        <x:fgColor rgb="FFF2F2F2"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="3">
     <x:border/>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9E2EC"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9E2EC"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9E2EC"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9E2EC"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE9EDF2"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE9EDF2"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE9EDF2"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE9EDF2"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="6">
+  <x:cellXfs count="10">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -55,8 +88,18 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -260,188 +303,188 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="86" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="76" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="145" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="96" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="125" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="255" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="105" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="92" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="120" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="240" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="100" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="255" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="25" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+    <x:row r="1" ht="22" customHeight="1">
+      <x:c r="A1" s="5" t="str">
         <x:v>Excel 行号</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="5" t="str">
         <x:v>订单编号</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="5" t="str">
         <x:v>客户姓名</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="5" t="str">
         <x:v>手机号</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="str">
+      <x:c r="E1" s="5" t="str">
         <x:v>短信内容</x:v>
       </x:c>
-      <x:c r="F1" s="4" t="str">
+      <x:c r="F1" s="5" t="str">
         <x:v>校验项</x:v>
       </x:c>
-      <x:c r="G1" s="4" t="str">
+      <x:c r="G1" s="5" t="str">
         <x:v>问题原因</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="5" t="n">
+    <x:row r="2" ht="26" customHeight="1">
+      <x:c r="A2" s="9" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="str"/>
-      <x:c r="C2" s="5" t="str">
+      <x:c r="B2" s="9" t="str"/>
+      <x:c r="C2" s="9" t="str">
         <x:v>张三</x:v>
       </x:c>
-      <x:c r="D2" s="5" t="str">
+      <x:c r="D2" s="9" t="str">
         <x:v>13800138000</x:v>
       </x:c>
-      <x:c r="E2" s="5" t="str">
+      <x:c r="E2" s="9" t="str">
         <x:v>【债转通知】请及时处理。</x:v>
       </x:c>
-      <x:c r="F2" s="5" t="str">
-        <x:v>必填字段</x:v>
-      </x:c>
-      <x:c r="G2" s="5" t="str">
+      <x:c r="F2" s="9" t="str">
+        <x:v>必填字段</x:v>
+      </x:c>
+      <x:c r="G2" s="9" t="str">
         <x:v>订单编号为空</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="5" t="n">
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="9" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B3" s="5" t="str">
+      <x:c r="B3" s="9" t="str">
         <x:v>SO20260805002</x:v>
       </x:c>
-      <x:c r="C3" s="5" t="str"/>
-      <x:c r="D3" s="5" t="str">
+      <x:c r="C3" s="9" t="str"/>
+      <x:c r="D3" s="9" t="str">
         <x:v>13900139000</x:v>
       </x:c>
-      <x:c r="E3" s="5" t="str">
+      <x:c r="E3" s="9" t="str">
         <x:v>【债转通知】请及时处理。</x:v>
       </x:c>
-      <x:c r="F3" s="5" t="str">
-        <x:v>必填字段</x:v>
-      </x:c>
-      <x:c r="G3" s="5" t="str">
+      <x:c r="F3" s="9" t="str">
+        <x:v>必填字段</x:v>
+      </x:c>
+      <x:c r="G3" s="9" t="str">
         <x:v>客户姓名为空</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="5" t="n">
+    <x:row r="4" ht="26" customHeight="1">
+      <x:c r="A4" s="9" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="str">
+      <x:c r="B4" s="9" t="str">
         <x:v>SO20260805003</x:v>
       </x:c>
-      <x:c r="C4" s="5" t="str">
+      <x:c r="C4" s="9" t="str">
         <x:v>李四</x:v>
       </x:c>
-      <x:c r="D4" s="5" t="str"/>
-      <x:c r="E4" s="5" t="str">
+      <x:c r="D4" s="9" t="str"/>
+      <x:c r="E4" s="9" t="str">
         <x:v>【债转通知】请及时处理。</x:v>
       </x:c>
-      <x:c r="F4" s="5" t="str">
-        <x:v>必填字段</x:v>
-      </x:c>
-      <x:c r="G4" s="5" t="str">
+      <x:c r="F4" s="9" t="str">
+        <x:v>必填字段</x:v>
+      </x:c>
+      <x:c r="G4" s="9" t="str">
         <x:v>手机号为空</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="5" t="n">
+    <x:row r="5" ht="26" customHeight="1">
+      <x:c r="A5" s="9" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="str">
+      <x:c r="B5" s="9" t="str">
         <x:v>SO20260805004</x:v>
       </x:c>
-      <x:c r="C5" s="5" t="str">
+      <x:c r="C5" s="9" t="str">
         <x:v>王五</x:v>
       </x:c>
-      <x:c r="D5" s="5" t="str">
+      <x:c r="D5" s="9" t="str">
         <x:v>13700137000</x:v>
       </x:c>
-      <x:c r="E5" s="5" t="str"/>
-      <x:c r="F5" s="5" t="str">
-        <x:v>必填字段</x:v>
-      </x:c>
-      <x:c r="G5" s="5" t="str">
+      <x:c r="E5" s="9" t="str"/>
+      <x:c r="F5" s="9" t="str">
+        <x:v>必填字段</x:v>
+      </x:c>
+      <x:c r="G5" s="9" t="str">
         <x:v>短信内容为空</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="5" t="n">
+    <x:row r="6" ht="26" customHeight="1">
+      <x:c r="A6" s="9" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="str">
+      <x:c r="B6" s="9" t="str">
         <x:v>SO20260805005</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="str">
+      <x:c r="C6" s="9" t="str">
         <x:v>赵六</x:v>
       </x:c>
-      <x:c r="D6" s="5" t="str">
+      <x:c r="D6" s="9" t="str">
         <x:v>13600136000</x:v>
       </x:c>
-      <x:c r="E6" s="5" t="str">
+      <x:c r="E6" s="9" t="str">
         <x:v>【债转通知】请及时处理。</x:v>
       </x:c>
-      <x:c r="F6" s="5" t="str">
+      <x:c r="F6" s="9" t="str">
         <x:v>订单状态</x:v>
       </x:c>
-      <x:c r="G6" s="5" t="str">
+      <x:c r="G6" s="9" t="str">
         <x:v>订单已结清</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="5" t="n">
+    <x:row r="7" ht="26" customHeight="1">
+      <x:c r="A7" s="9" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="str">
+      <x:c r="B7" s="9" t="str">
         <x:v>SO20260805006</x:v>
       </x:c>
-      <x:c r="C7" s="5" t="str">
+      <x:c r="C7" s="9" t="str">
         <x:v>钱七</x:v>
       </x:c>
-      <x:c r="D7" s="5" t="str">
+      <x:c r="D7" s="9" t="str">
         <x:v>12345678901</x:v>
       </x:c>
-      <x:c r="E7" s="5" t="str">
+      <x:c r="E7" s="9" t="str">
         <x:v>【债转通知】请及时处理。</x:v>
       </x:c>
-      <x:c r="F7" s="5" t="str">
+      <x:c r="F7" s="9" t="str">
         <x:v>手机号</x:v>
       </x:c>
-      <x:c r="G7" s="5" t="str">
+      <x:c r="G7" s="9" t="str">
         <x:v>手机号格式错误</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="5" t="n">
+    <x:row r="8" ht="26" customHeight="1">
+      <x:c r="A8" s="9" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="str">
+      <x:c r="B8" s="9" t="str">
         <x:v>SO20260805007</x:v>
       </x:c>
-      <x:c r="C8" s="5" t="str">
+      <x:c r="C8" s="9" t="str">
         <x:v>孙八</x:v>
       </x:c>
-      <x:c r="D8" s="5" t="str">
+      <x:c r="D8" s="9" t="str">
         <x:v>13500135000</x:v>
       </x:c>
-      <x:c r="E8" s="5" t="str">
+      <x:c r="E8" s="9" t="str">
         <x:v>【债转通知】请及时处理。</x:v>
       </x:c>
-      <x:c r="F8" s="5" t="str">
+      <x:c r="F8" s="9" t="str">
         <x:v>重复触达</x:v>
       </x:c>
-      <x:c r="G8" s="5" t="str">
+      <x:c r="G8" s="9" t="str">
         <x:v>订单编号、客户姓名、手机号、短信内容四项完全一致</x:v>
       </x:c>
     </x:row>
@@ -454,146 +497,146 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="160" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="105" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="130" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="145" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="100" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="125" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="255" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="170" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="165" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="25" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+    <x:row r="1" ht="22" customHeight="1">
+      <x:c r="A1" s="5" t="str">
         <x:v>类型编码</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="5" t="str">
         <x:v>校验项</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="5" t="str">
         <x:v>错误场景</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="5" t="str">
         <x:v>判定规则</x:v>
       </x:c>
-      <x:c r="E1" s="4" t="str">
+      <x:c r="E1" s="5" t="str">
         <x:v>处理结果</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="5" t="str">
+    <x:row r="2" ht="26" customHeight="1">
+      <x:c r="A2" s="9" t="str">
         <x:v>REQUIRED_ORDER_NO</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="str">
-        <x:v>必填字段</x:v>
-      </x:c>
-      <x:c r="C2" s="5" t="str">
+      <x:c r="B2" s="9" t="str">
+        <x:v>必填字段</x:v>
+      </x:c>
+      <x:c r="C2" s="9" t="str">
         <x:v>订单编号为空</x:v>
       </x:c>
-      <x:c r="D2" s="5" t="str">
+      <x:c r="D2" s="9" t="str">
         <x:v>订单编号未填写或仅包含空格</x:v>
       </x:c>
-      <x:c r="E2" s="5" t="str">
+      <x:c r="E2" s="9" t="str">
         <x:v>该行不进入发送队列</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="5" t="str">
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="9" t="str">
         <x:v>REQUIRED_NAME</x:v>
       </x:c>
-      <x:c r="B3" s="5" t="str">
-        <x:v>必填字段</x:v>
-      </x:c>
-      <x:c r="C3" s="5" t="str">
+      <x:c r="B3" s="9" t="str">
+        <x:v>必填字段</x:v>
+      </x:c>
+      <x:c r="C3" s="9" t="str">
         <x:v>客户姓名为空</x:v>
       </x:c>
-      <x:c r="D3" s="5" t="str">
+      <x:c r="D3" s="9" t="str">
         <x:v>客户姓名未填写或仅包含空格</x:v>
       </x:c>
-      <x:c r="E3" s="5" t="str">
+      <x:c r="E3" s="9" t="str">
         <x:v>该行不进入发送队列</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="5" t="str">
+    <x:row r="4" ht="26" customHeight="1">
+      <x:c r="A4" s="9" t="str">
         <x:v>REQUIRED_PHONE</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="str">
-        <x:v>必填字段</x:v>
-      </x:c>
-      <x:c r="C4" s="5" t="str">
+      <x:c r="B4" s="9" t="str">
+        <x:v>必填字段</x:v>
+      </x:c>
+      <x:c r="C4" s="9" t="str">
         <x:v>手机号为空</x:v>
       </x:c>
-      <x:c r="D4" s="5" t="str">
+      <x:c r="D4" s="9" t="str">
         <x:v>手机号未填写或仅包含空格</x:v>
       </x:c>
-      <x:c r="E4" s="5" t="str">
+      <x:c r="E4" s="9" t="str">
         <x:v>该行不进入发送队列</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="5" t="str">
+    <x:row r="5" ht="26" customHeight="1">
+      <x:c r="A5" s="9" t="str">
         <x:v>REQUIRED_MESSAGE</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="str">
-        <x:v>必填字段</x:v>
-      </x:c>
-      <x:c r="C5" s="5" t="str">
+      <x:c r="B5" s="9" t="str">
+        <x:v>必填字段</x:v>
+      </x:c>
+      <x:c r="C5" s="9" t="str">
         <x:v>短信内容为空</x:v>
       </x:c>
-      <x:c r="D5" s="5" t="str">
+      <x:c r="D5" s="9" t="str">
         <x:v>短信内容未填写或仅包含空格</x:v>
       </x:c>
-      <x:c r="E5" s="5" t="str">
+      <x:c r="E5" s="9" t="str">
         <x:v>该行不进入发送队列</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="5" t="str">
+    <x:row r="6" ht="26" customHeight="1">
+      <x:c r="A6" s="9" t="str">
         <x:v>ORDER_SETTLED</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="str">
+      <x:c r="B6" s="9" t="str">
         <x:v>订单状态</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="str">
+      <x:c r="C6" s="9" t="str">
         <x:v>订单已结清</x:v>
       </x:c>
-      <x:c r="D6" s="5" t="str">
+      <x:c r="D6" s="9" t="str">
         <x:v>订单实时状态为已结清</x:v>
       </x:c>
-      <x:c r="E6" s="5" t="str">
+      <x:c r="E6" s="9" t="str">
         <x:v>不允许发送</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="5" t="str">
+    <x:row r="7" ht="26" customHeight="1">
+      <x:c r="A7" s="9" t="str">
         <x:v>PHONE_INVALID</x:v>
       </x:c>
-      <x:c r="B7" s="5" t="str">
+      <x:c r="B7" s="9" t="str">
         <x:v>手机号</x:v>
       </x:c>
-      <x:c r="C7" s="5" t="str">
+      <x:c r="C7" s="9" t="str">
         <x:v>手机号格式错误</x:v>
       </x:c>
-      <x:c r="D7" s="5" t="str">
+      <x:c r="D7" s="9" t="str">
         <x:v>不符合 11 位中国大陆手机号规范</x:v>
       </x:c>
-      <x:c r="E7" s="5" t="str">
+      <x:c r="E7" s="9" t="str">
         <x:v>该行不进入发送队列</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="5" t="str">
+    <x:row r="8" ht="26" customHeight="1">
+      <x:c r="A8" s="9" t="str">
         <x:v>DUPLICATE_TOUCH</x:v>
       </x:c>
-      <x:c r="B8" s="5" t="str">
+      <x:c r="B8" s="9" t="str">
         <x:v>重复触达</x:v>
       </x:c>
-      <x:c r="C8" s="5" t="str">
+      <x:c r="C8" s="9" t="str">
         <x:v>重复触达</x:v>
       </x:c>
-      <x:c r="D8" s="5" t="str">
+      <x:c r="D8" s="9" t="str">
         <x:v>订单编号、客户姓名、手机号、短信内容四项完全一致</x:v>
       </x:c>
-      <x:c r="E8" s="5" t="str">
+      <x:c r="E8" s="9" t="str">
         <x:v>该行不进入发送队列</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
style: compact sms error workbook columns
</commit_message>
<xml_diff>
--- a/debt-transfer-sms-notification/assets/短信通知_导入错误明细.xlsx
+++ b/debt-transfer-sms-notification/assets/短信通知_导入错误明细.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="错误数据明细" sheetId="1" r:id="R4e0d7ae102d04a58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="错误类型说明" sheetId="2" r:id="Rcb256ac651d44035"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="错误数据明细" sheetId="1" r:id="Rc417e7b5ec7f423d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="错误类型说明" sheetId="2" r:id="Rcbbbecd25fec4a91"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -303,13 +303,13 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="76" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="145" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="92" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="120" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="240" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="100" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="255" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="7.21999979019165" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="8.890000343322754" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="11.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="21.110000610351562" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="22" customHeight="1">
@@ -497,11 +497,11 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="145" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="100" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="125" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="255" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="165" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="15" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="11.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22.780000686645508" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14.4399995803833" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="22" customHeight="1">

</xml_diff>

<commit_message>
style: widen sms error detail columns
</commit_message>
<xml_diff>
--- a/debt-transfer-sms-notification/assets/短信通知_导入错误明细.xlsx
+++ b/debt-transfer-sms-notification/assets/短信通知_导入错误明细.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="错误数据明细" sheetId="1" r:id="Rc417e7b5ec7f423d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="错误类型说明" sheetId="2" r:id="Rcbbbecd25fec4a91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="错误数据明细" sheetId="1" r:id="R85d3e3b991a34c59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="错误类型说明" sheetId="2" r:id="R6488aabcd05340dd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -304,12 +304,12 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="7.21999979019165" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="11.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="8.890000343322754" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="11.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18.889999389648438" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="9.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="21.110000610351562" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="26.670000076293945" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="22" customHeight="1">

</xml_diff>